<commit_message>
Update handle-database.xlsx after carousel run
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/handle-database.xlsx
+++ b/data/carousel-workflow/handle-database.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -520,6 +520,654 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Robert Sutton</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Stanford University</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/bobsutton1/</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>@work_matters</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>The No Asshole Rule author</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Kim Scott</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Radical Candor</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/kimm4/</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>@kimballscott</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>@kimmalonescott</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Radical Candor author</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Amy Edmondson</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Harvard Business School</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>@AmyCEdmondson</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>@amycedmondson.bsky.social</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Psychological safety researcher</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Simon Sinek</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/simonsinek/</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>@simonsinek</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>@simonsinek</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Simon Sinek</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Start With Why author</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Patrick Lencioni</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>The Table Group</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/patrick-lencioni-orghealth/</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>@patricklencioni</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>@patricklencioniofficial</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>@PatrickLencioniOfficial</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Working Genius, Five Dysfunctions author</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Liz Wiseman</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>The Wiseman Group</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/lizwiseman</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>@LizWiseman</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>@bylizwiseman</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Multipliers author</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Tessa West</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>NYU</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/tessa-west-129b51131/</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>@TessaWestNYU</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Jerks at Work author</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Adam Grant</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Wharton</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/adammgrant/</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>@AdamMGrant</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>@adamgrant</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>@adamgrant</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Give and Take author</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Dave Bailey</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>CEO Coach</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/davesuperman/</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>@davesuperman</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>CEO coach</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Kathryn Landis</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Executive Coach</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/kathrynlandis/</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Executive coach, LinkedIn active</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Tim Duggan</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Author</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/timduggan1</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>@tim_duggan</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Australian workplace culture author</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Achim Nowak</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Executive Coach</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/achimnowak/</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>@AchimNowak</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Executive coach</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Reed Hastings</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Netflix</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/reedhastings</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>@reedhastings</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Netflix co-founder</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:N1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update handle-database.xlsx after carousel run 2026-03-25
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/handle-database.xlsx
+++ b/data/carousel-workflow/handle-database.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N50"/>
+  <dimension ref="A1:N58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2713,6 +2713,442 @@
         </is>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Jeff Bezos</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr"/>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>@JeffBezos</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>@jeffbezos</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="inlineStr"/>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr"/>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>No LinkedIn profile</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Daniel Pink</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Author</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/danielpink</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>@DanielPink</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>@danielpink</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr"/>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>@danielhpink</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr"/>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Columbia Business School</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Business School</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>columbia-business-school</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>@Columbia_Biz</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>@columbia_biz</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>@columbia_biz</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>@columbia_biz</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>@columbiabusiness.bsky.social</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>facebook.com/columbiabusiness</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Harvard Business School</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Business School</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>harvard-business-school</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>@HarvardHBS</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>@harvardhbs</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>@harvardhbs</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>@harvardhbs</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>@harvardhbs.bsky.social</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>facebook.com/harvardbusinessschool</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Deloitte</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Consulting</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>deloitte</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>@Deloitte</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>@deloitte</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>@deloitte</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr"/>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>facebook.com/deloitte</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr"/>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>McKinsey &amp; Company</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Consulting</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>mckinsey</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>@McKinsey</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr"/>
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" t="inlineStr"/>
+      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="inlineStr"/>
+      <c r="J56" t="inlineStr"/>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Bain &amp; Company</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Consulting</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>bain-and-company</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>@BainandCompany</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>@bainandcompany</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr"/>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>facebook.com/bainandcompany</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr"/>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>amazon</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>@Amazon</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>@amazon</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>@amazon</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>facebook.com/Amazon</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:N1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update handle-database.xlsx after WG-Hiring carousel run 2026-03-25
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/handle-database.xlsx
+++ b/data/carousel-workflow/handle-database.xlsx
@@ -2724,7 +2724,6 @@
           <t>Amazon</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr"/>
       <c r="D51" t="inlineStr">
         <is>
           <t>@JeffBezos</t>
@@ -2735,11 +2734,6 @@
           <t>@jeffbezos</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr"/>
-      <c r="G51" t="inlineStr"/>
-      <c r="H51" t="inlineStr"/>
-      <c r="I51" t="inlineStr"/>
-      <c r="J51" t="inlineStr"/>
       <c r="K51" t="inlineStr">
         <is>
           <t>2026-03-25</t>
@@ -2787,15 +2781,11 @@
           <t>@danielpink</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr"/>
-      <c r="G52" t="inlineStr"/>
-      <c r="H52" t="inlineStr"/>
       <c r="I52" t="inlineStr">
         <is>
           <t>@danielhpink</t>
         </is>
       </c>
-      <c r="J52" t="inlineStr"/>
       <c r="K52" t="inlineStr">
         <is>
           <t>2026-03-25</t>
@@ -2811,7 +2801,6 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="N52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2859,7 +2848,6 @@
           <t>facebook.com/columbiabusiness</t>
         </is>
       </c>
-      <c r="J53" t="inlineStr"/>
       <c r="K53" t="inlineStr">
         <is>
           <t>2026-03-25</t>
@@ -2875,7 +2863,6 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="N53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2923,7 +2910,6 @@
           <t>facebook.com/harvardbusinessschool</t>
         </is>
       </c>
-      <c r="J54" t="inlineStr"/>
       <c r="K54" t="inlineStr">
         <is>
           <t>2026-03-25</t>
@@ -2939,7 +2925,6 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="N54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2972,14 +2957,11 @@
           <t>@deloitte</t>
         </is>
       </c>
-      <c r="G55" t="inlineStr"/>
-      <c r="H55" t="inlineStr"/>
       <c r="I55" t="inlineStr">
         <is>
           <t>facebook.com/deloitte</t>
         </is>
       </c>
-      <c r="J55" t="inlineStr"/>
       <c r="K55" t="inlineStr">
         <is>
           <t>2026-03-25</t>
@@ -2995,7 +2977,6 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="N55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3018,12 +2999,6 @@
           <t>@McKinsey</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr"/>
-      <c r="F56" t="inlineStr"/>
-      <c r="G56" t="inlineStr"/>
-      <c r="H56" t="inlineStr"/>
-      <c r="I56" t="inlineStr"/>
-      <c r="J56" t="inlineStr"/>
       <c r="K56" t="inlineStr">
         <is>
           <t>2026-03-25</t>
@@ -3039,7 +3014,6 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="N56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3067,15 +3041,11 @@
           <t>@bainandcompany</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr"/>
-      <c r="G57" t="inlineStr"/>
-      <c r="H57" t="inlineStr"/>
       <c r="I57" t="inlineStr">
         <is>
           <t>facebook.com/bainandcompany</t>
         </is>
       </c>
-      <c r="J57" t="inlineStr"/>
       <c r="K57" t="inlineStr">
         <is>
           <t>2026-03-25</t>
@@ -3091,7 +3061,6 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="N57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3119,19 +3088,16 @@
           <t>@amazon</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
           <t>@amazon</t>
         </is>
       </c>
-      <c r="H58" t="inlineStr"/>
       <c r="I58" t="inlineStr">
         <is>
           <t>facebook.com/Amazon</t>
         </is>
       </c>
-      <c r="J58" t="inlineStr"/>
       <c r="K58" t="inlineStr">
         <is>
           <t>2026-03-25</t>
@@ -3147,7 +3113,6 @@
           <t>ACTIVE</t>
         </is>
       </c>
-      <c r="N58" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:N1"/>

</xml_diff>

<commit_message>
Update handle-database.xlsx after sleep-leadership carousel run
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/handle-database.xlsx
+++ b/data/carousel-workflow/handle-database.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N58"/>
+  <dimension ref="A1:N65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3114,6 +3114,330 @@
         </is>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Christopher M. Barnes</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>University of Washington</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>@chris24barnes</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>Sleep &amp; leadership researcher. X handle LIKELY.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Dr. Els van der Helm</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>@elsonsleep</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>@drelsvanderhelm</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>Sleep neuroscientist. Handles LIKELY.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Dr. Sophie Bostock</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>@drsophiebostock</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>@drsophiebostock</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>@drsophiebostock</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>@drsophiebostock</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>Sleep scientist. Handles LIKELY.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Matthew Walker</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>@sleepdiplomat</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>@drmattwalker</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>@sleepdiplomat</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>@sleepdiplomat</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>@sleepdiplomat</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>Neuroscientist, Why We Sleep author. VERIFIED.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Dr. Shelby Harris</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>@SleepDocShelby</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>@SleepDocShelby</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>@sleepdocshelby</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>Behavioral sleep medicine. VERIFIED.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Arianna Huffington</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Thrive Global</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>@ariannahuff</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>@ariannahuff</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>@ariannahuff</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Arianna Huffington</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>@ariannahuff.bsky.social</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>AriannaHuffington</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>Thrive Global founder. VERIFIED.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Nick Littlehales</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>@SportSleepCoach</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>@sportsleepcoach</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>@sportsleepcoach</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>sportsleepcoach</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>Elite sport sleep coach. R90 method. LIKELY.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:N1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update handle-database.xlsx after loneliness carousel run 2026-03-25
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/handle-database.xlsx
+++ b/data/carousel-workflow/handle-database.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N65"/>
+  <dimension ref="A1:N72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3438,6 +3438,236 @@
         </is>
       </c>
     </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Chester Elton</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr"/>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>@chesterelton</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>@chesterelton</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr"/>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" t="inlineStr"/>
+      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr"/>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>Leadership loneliness blog - author of Leading with Gratitude</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Ed Batista</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr"/>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>@edbatista</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr"/>
+      <c r="H67" t="inlineStr"/>
+      <c r="I67" t="inlineStr"/>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>Leadership loneliness blog - executive coach, Stanford lecturer</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Vivek Murthy</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr"/>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>@vivabornerthy</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="inlineStr"/>
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" t="inlineStr"/>
+      <c r="H68" t="inlineStr"/>
+      <c r="I68" t="inlineStr"/>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>Leadership loneliness blog - former US Surgeon General, loneliness epidemic</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Julianne Holt-Lunstad</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr"/>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>@jholtlunstad</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="inlineStr"/>
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" t="inlineStr"/>
+      <c r="H69" t="inlineStr"/>
+      <c r="I69" t="inlineStr"/>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>LIKELY</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>Leadership loneliness blog - BYU researcher on social connections and health</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Nick Jonsson</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr"/>
+      <c r="C70" t="inlineStr"/>
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="inlineStr"/>
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="inlineStr"/>
+      <c r="H70" t="inlineStr"/>
+      <c r="I70" t="inlineStr"/>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>Leadership loneliness blog - author of Executive Loneliness</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Morra Aarons-Mele</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr"/>
+      <c r="C71" t="inlineStr"/>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="inlineStr"/>
+      <c r="F71" t="inlineStr"/>
+      <c r="G71" t="inlineStr"/>
+      <c r="H71" t="inlineStr"/>
+      <c r="I71" t="inlineStr"/>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>Leadership loneliness blog - author of The Anxious Achiever</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Jerry Colonna</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr"/>
+      <c r="C72" t="inlineStr"/>
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="inlineStr"/>
+      <c r="F72" t="inlineStr"/>
+      <c r="G72" t="inlineStr"/>
+      <c r="H72" t="inlineStr"/>
+      <c r="I72" t="inlineStr"/>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>Leadership loneliness blog - CEO coach, author of Reboot</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:N1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update handle-database.xlsx after caring-hurts-leadership run
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/handle-database.xlsx
+++ b/data/carousel-workflow/handle-database.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N72"/>
+  <dimension ref="A1:N77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3444,7 +3444,6 @@
           <t>Chester Elton</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr"/>
       <c r="C66" t="inlineStr">
         <is>
           <t>@chesterelton</t>
@@ -3455,11 +3454,6 @@
           <t>@chesterelton</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr"/>
-      <c r="F66" t="inlineStr"/>
-      <c r="G66" t="inlineStr"/>
-      <c r="H66" t="inlineStr"/>
-      <c r="I66" t="inlineStr"/>
       <c r="J66" t="inlineStr">
         <is>
           <t>2026-03-25</t>
@@ -3482,18 +3476,11 @@
           <t>Ed Batista</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr"/>
       <c r="C67" t="inlineStr">
         <is>
           <t>@edbatista</t>
         </is>
       </c>
-      <c r="D67" t="inlineStr"/>
-      <c r="E67" t="inlineStr"/>
-      <c r="F67" t="inlineStr"/>
-      <c r="G67" t="inlineStr"/>
-      <c r="H67" t="inlineStr"/>
-      <c r="I67" t="inlineStr"/>
       <c r="J67" t="inlineStr">
         <is>
           <t>2026-03-25</t>
@@ -3516,18 +3503,11 @@
           <t>Vivek Murthy</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr"/>
       <c r="C68" t="inlineStr">
         <is>
           <t>@vivabornerthy</t>
         </is>
       </c>
-      <c r="D68" t="inlineStr"/>
-      <c r="E68" t="inlineStr"/>
-      <c r="F68" t="inlineStr"/>
-      <c r="G68" t="inlineStr"/>
-      <c r="H68" t="inlineStr"/>
-      <c r="I68" t="inlineStr"/>
       <c r="J68" t="inlineStr">
         <is>
           <t>2026-03-25</t>
@@ -3550,18 +3530,11 @@
           <t>Julianne Holt-Lunstad</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr"/>
       <c r="C69" t="inlineStr">
         <is>
           <t>@jholtlunstad</t>
         </is>
       </c>
-      <c r="D69" t="inlineStr"/>
-      <c r="E69" t="inlineStr"/>
-      <c r="F69" t="inlineStr"/>
-      <c r="G69" t="inlineStr"/>
-      <c r="H69" t="inlineStr"/>
-      <c r="I69" t="inlineStr"/>
       <c r="J69" t="inlineStr">
         <is>
           <t>2026-03-25</t>
@@ -3584,14 +3557,6 @@
           <t>Nick Jonsson</t>
         </is>
       </c>
-      <c r="B70" t="inlineStr"/>
-      <c r="C70" t="inlineStr"/>
-      <c r="D70" t="inlineStr"/>
-      <c r="E70" t="inlineStr"/>
-      <c r="F70" t="inlineStr"/>
-      <c r="G70" t="inlineStr"/>
-      <c r="H70" t="inlineStr"/>
-      <c r="I70" t="inlineStr"/>
       <c r="J70" t="inlineStr">
         <is>
           <t>2026-03-25</t>
@@ -3614,14 +3579,6 @@
           <t>Morra Aarons-Mele</t>
         </is>
       </c>
-      <c r="B71" t="inlineStr"/>
-      <c r="C71" t="inlineStr"/>
-      <c r="D71" t="inlineStr"/>
-      <c r="E71" t="inlineStr"/>
-      <c r="F71" t="inlineStr"/>
-      <c r="G71" t="inlineStr"/>
-      <c r="H71" t="inlineStr"/>
-      <c r="I71" t="inlineStr"/>
       <c r="J71" t="inlineStr">
         <is>
           <t>2026-03-25</t>
@@ -3644,14 +3601,6 @@
           <t>Jerry Colonna</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr"/>
-      <c r="C72" t="inlineStr"/>
-      <c r="D72" t="inlineStr"/>
-      <c r="E72" t="inlineStr"/>
-      <c r="F72" t="inlineStr"/>
-      <c r="G72" t="inlineStr"/>
-      <c r="H72" t="inlineStr"/>
-      <c r="I72" t="inlineStr"/>
       <c r="J72" t="inlineStr">
         <is>
           <t>2026-03-25</t>
@@ -3665,6 +3614,176 @@
       <c r="L72" t="inlineStr">
         <is>
           <t>Leadership loneliness blog - CEO coach, author of Reboot</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Henry Cloud</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Boundaries/DrCloud.com</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>@DrHenryCloud</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>DrHenryCloud</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="N73" t="inlineStr">
+        <is>
+          <t>Boundaries author</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>John Townsend</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Townsend Institute</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>@drjohntownsend</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="N74" t="inlineStr">
+        <is>
+          <t>Boundaries co-author</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Tania Singer</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Max Planck Institute</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>INACTIVE</t>
+        </is>
+      </c>
+      <c r="N75" t="inlineStr">
+        <is>
+          <t>Neuroscience researcher, minimal social media</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>David Morrison</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Retired Australian Army</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>INACTIVE</t>
+        </is>
+      </c>
+      <c r="N76" t="inlineStr">
+        <is>
+          <t>Former Australian Army Chief, no social accounts</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Edwin Friedman</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="M77" t="inlineStr">
+        <is>
+          <t>DECEASED</t>
+        </is>
+      </c>
+      <c r="N77" t="inlineStr">
+        <is>
+          <t>Died 1996. Family systems leadership author.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update handle-database.xlsx after carousel run - Craig Groeschel Podcast
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/handle-database.xlsx
+++ b/data/carousel-workflow/handle-database.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N77"/>
+  <dimension ref="A1:N79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3787,6 +3787,130 @@
         </is>
       </c>
     </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Craig Groeschel</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Life.Church</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>craig-groeschel-11463a112</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>@craiggroeschel</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>@craiggroeschel</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>@craiggroeschel</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>@craiggroeschel</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>@craiggroeschel</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>craiggroeschel</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="N78" t="inlineStr">
+        <is>
+          <t>Founder Life.Church. Threads LIKELY. X possibly inactive. Bluesky NOT FOUND.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Life.Church</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Life.Church</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>@life.church</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>@lifechurch</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>@life.church</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>life.church</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="N79" t="inlineStr">
+        <is>
+          <t>Church org. Tagged on IG and FB.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:N1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update handle-database.xlsx after ASBA testimonial carousel run
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/handle-database.xlsx
+++ b/data/carousel-workflow/handle-database.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N79"/>
+  <dimension ref="A1:N81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3911,6 +3911,80 @@
         </is>
       </c>
     </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>ASBA Limited</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>ASBA</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>ASBALtd</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="N80" t="inlineStr">
+        <is>
+          <t>Peak body for independent school business managers in Australia/NZ. CEO: Kathy Dickson.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Kathy Dickson</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>ASBA</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/kathy-dickson</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="M81" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="N81" t="inlineStr">
+        <is>
+          <t>CEO of ASBA. LinkedIn only (personal profile, cannot tag via API).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:N1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update handle database - Topic 2 Jocko/Leif
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/handle-database.xlsx
+++ b/data/carousel-workflow/handle-database.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N81"/>
+  <dimension ref="A1:N83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3985,6 +3985,105 @@
         </is>
       </c>
     </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Jocko Willink</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Echelon Front</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>@jockowillink</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>@jockowillink</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>@jocko_willink</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Jocko Willink</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>Jocko Willink</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="N82" t="inlineStr">
+        <is>
+          <t>Extreme Ownership co-author, Navy SEAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Leif Babin</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Echelon Front</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/leif-babin-2a43b631/</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>@leifbabin</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="M83" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="N83" t="inlineStr">
+        <is>
+          <t>Extreme Ownership co-author, Navy SEAL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:N1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update handle-database - Topic 4 Learning Leader
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/handle-database.xlsx
+++ b/data/carousel-workflow/handle-database.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N83"/>
+  <dimension ref="A1:N84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -4084,6 +4084,48 @@
         </is>
       </c>
     </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Ryan Hawk</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>ryanhawk12</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>@RyanHawk12</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>@ryanhawk12</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>TheLearningLeaderShow</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>Podcast host, author, speaker</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:N1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update handle-database.xlsx - Topic 1: Edward Amey testimonial
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/handle-database.xlsx
+++ b/data/carousel-workflow/handle-database.xlsx
@@ -18,7 +18,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -59,11 +61,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N84"/>
+  <dimension ref="A1:N85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -4126,6 +4129,39 @@
         </is>
       </c>
     </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Edward Amey</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Jay Nolan Community Services</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>edward-r-amey-ms-5280aa5</t>
+        </is>
+      </c>
+      <c r="K85" s="2" t="n">
+        <v>46108</v>
+      </c>
+      <c r="L85" s="2" t="n">
+        <v>46108</v>
+      </c>
+      <c r="M85" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="N85" t="inlineStr">
+        <is>
+          <t>CEO Jay Nolan Community Services. LinkedIn verified. No other social media found.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:N1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update handle database - Crucial Conversations
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/handle-database.xlsx
+++ b/data/carousel-workflow/handle-database.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N85"/>
+  <dimension ref="A1:N86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -4162,6 +4162,48 @@
         </is>
       </c>
     </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Crucial Learning (VitalSmarts)</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Crucial Learning</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>company/crucial-learning</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>@VitalSmarts</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="N86" t="inlineStr">
+        <is>
+          <t>Publishers of Crucial Conversations. Formerly VitalSmarts.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:N1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update handle-database: Add John Maxwell
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/handle-database.xlsx
+++ b/data/carousel-workflow/handle-database.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N87"/>
+  <dimension ref="A1:N88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -4261,6 +4261,65 @@
         </is>
       </c>
     </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>John Maxwell</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>The John Maxwell Company</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>johncmaxwell</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>@JohnCMaxwell</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>@johncmaxwell</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>@johncmaxwell</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr"/>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>johnmaxwell</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr"/>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="M88" t="inlineStr">
+        <is>
+          <t>Major leadership figure. X/Twitter and Instagram verified. No confirmed Bluesky or Threads.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:N1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update handle-database.xlsx — Topic 4 coaching-for-leaders
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/handle-database.xlsx
+++ b/data/carousel-workflow/handle-database.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N88"/>
+  <dimension ref="A1:N89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -4318,6 +4318,48 @@
         </is>
       </c>
     </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Dave Stachowiak</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Host, Coaching for Leaders podcast</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Coaching for Leaders</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>davestachowiak</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>@davestachowiak</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="M89" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N89" t="inlineStr">
+        <is>
+          <t>X: VERIFIED, LinkedIn: VERIFIED. No IG/TikTok/YT/Threads/Bluesky found.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:N1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update handle-database.xlsx - Topic 1 Ian Cumming testimonial
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/handle-database.xlsx
+++ b/data/carousel-workflow/handle-database.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N89"/>
+  <dimension ref="A1:N90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -4360,6 +4360,43 @@
         </is>
       </c>
     </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Ian Cumming</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>SU Australia</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>ian-cumming-gaicd-157b885b</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="N90" t="inlineStr">
+        <is>
+          <t>GAICD, Group Director Operations, MBA. Only LinkedIn found.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:N1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update handle database - Topic 1 GLS Podcast
</commit_message>
<xml_diff>
--- a/data/carousel-workflow/handle-database.xlsx
+++ b/data/carousel-workflow/handle-database.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N90"/>
+  <dimension ref="A1:N92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -4397,6 +4397,82 @@
         </is>
       </c>
     </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>David Ashcraft</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Global Leadership Network</t>
+        </is>
+      </c>
+      <c r="K91" s="2" t="n">
+        <v>46110</v>
+      </c>
+      <c r="L91" s="2" t="n">
+        <v>46110</v>
+      </c>
+      <c r="M91" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="N91" t="inlineStr">
+        <is>
+          <t>GLS Podcast host</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Whitney Putnam</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Global Leadership Network</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>@glnsummit</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>@glnsummit</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>@glnsummit</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>Global Leadership Network</t>
+        </is>
+      </c>
+      <c r="K92" s="2" t="n">
+        <v>46110</v>
+      </c>
+      <c r="L92" s="2" t="n">
+        <v>46110</v>
+      </c>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="N92" t="inlineStr">
+        <is>
+          <t>GLS Podcast host</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:N1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>